<commit_message>
Update worklog_set1 template and adapt program mappings
</commit_message>
<xml_diff>
--- a/worklog_set1.xlsx
+++ b/worklog_set1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\worklog-automation-tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{947D7F54-58FB-489C-8C03-AD4ED608FD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF50BADD-B735-42D1-8431-507420BE410C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9540" yWindow="360" windowWidth="24735" windowHeight="15045" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4월" sheetId="20" r:id="rId1"/>
@@ -28,18 +28,12 @@
     <t>평생교육사업1 업무일지</t>
   </si>
   <si>
-    <t>일본어(초급)</t>
-  </si>
-  <si>
     <t>컴퓨터실</t>
   </si>
   <si>
     <t>모니터링</t>
   </si>
   <si>
-    <t>중국어(초급)</t>
-  </si>
-  <si>
     <t>생활한자</t>
   </si>
   <si>
@@ -56,9 +50,6 @@
   </si>
   <si>
     <t>한문서예3반</t>
-  </si>
-  <si>
-    <t>영어(중급)</t>
   </si>
   <si>
     <t>체어요가</t>
@@ -83,9 +74,6 @@
     <t>작품전시회</t>
   </si>
   <si>
-    <t>중국어(중급)</t>
-  </si>
-  <si>
     <t>만족도
 조사</t>
   </si>
@@ -99,12 +87,6 @@
     <t>수강신청</t>
   </si>
   <si>
-    <t>일본어(중급)</t>
-  </si>
-  <si>
-    <t>영어(초급)</t>
-  </si>
-  <si>
     <t>한글서예2반</t>
   </si>
   <si>
@@ -167,12 +149,6 @@
   </si>
   <si>
     <t>반장/강사 간담회</t>
-  </si>
-  <si>
-    <t>한글교실(중급)</t>
-  </si>
-  <si>
-    <t>한글교실(초급1)</t>
   </si>
   <si>
     <t>평생
@@ -190,9 +166,6 @@
     <t>프로그램 만족도 조사</t>
   </si>
   <si>
-    <t>한글교실(초급2)</t>
-  </si>
-  <si>
     <t>관장</t>
   </si>
   <si>
@@ -276,11 +249,6 @@
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
-    <t>특강  및
- 외부대회 참여지원</t>
-    <phoneticPr fontId="9" type="noConversion"/>
-  </si>
-  <si>
     <t>팝송영어</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
@@ -298,6 +266,47 @@
   </si>
   <si>
     <t>파워요가</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>영어 첫걸금</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>생활 영어</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>일본어 첫걸음</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>일본어 회화</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>중국어 첫걸음</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>중국어 회화</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>한글교실 초급</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>한글교실 중급</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>한글교실 고급</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>특강  및 
+외부대회 참여지원</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
@@ -618,7 +627,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -733,6 +742,153 @@
     <xf numFmtId="41" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -757,152 +913,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1458,126 +1470,126 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="33" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="76" t="s">
-        <v>15</v>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="77" t="s">
+        <v>12</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="I1" s="18" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="J1" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="K1" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="L1" s="17" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" s="33" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="76"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="79" t="s">
+        <v>53</v>
+      </c>
+      <c r="L2" s="59"/>
+    </row>
+    <row r="3" spans="1:12" s="33" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="61">
+        <v>46113</v>
+      </c>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="78"/>
+      <c r="K3" s="79"/>
+      <c r="L3" s="60"/>
+    </row>
+    <row r="4" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="63"/>
+      <c r="C4" s="66" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="67"/>
+      <c r="E4" s="68" t="s">
         <v>55</v>
       </c>
-      <c r="K1" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="L1" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" s="33" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="75"/>
-      <c r="B2" s="75"/>
-      <c r="C2" s="75"/>
-      <c r="D2" s="75"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="75"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="77"/>
-      <c r="I2" s="77"/>
-      <c r="J2" s="77"/>
-      <c r="K2" s="78" t="s">
-        <v>62</v>
-      </c>
-      <c r="L2" s="58"/>
-    </row>
-    <row r="3" spans="1:12" s="33" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="60">
-        <v>46113</v>
-      </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="76"/>
-      <c r="H3" s="77"/>
-      <c r="I3" s="77"/>
-      <c r="J3" s="77"/>
-      <c r="K3" s="78"/>
-      <c r="L3" s="59"/>
-    </row>
-    <row r="4" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="61" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" s="62"/>
-      <c r="C4" s="65" t="s">
-        <v>56</v>
-      </c>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67" t="s">
-        <v>64</v>
-      </c>
-      <c r="F4" s="68"/>
-      <c r="G4" s="69" t="s">
-        <v>74</v>
-      </c>
-      <c r="H4" s="70"/>
-      <c r="I4" s="69" t="s">
-        <v>72</v>
-      </c>
-      <c r="J4" s="70"/>
-      <c r="K4" s="71" t="s">
-        <v>59</v>
-      </c>
-      <c r="L4" s="72"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="70" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" s="71"/>
+      <c r="I4" s="70" t="s">
+        <v>63</v>
+      </c>
+      <c r="J4" s="71"/>
+      <c r="K4" s="72" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" s="73"/>
     </row>
     <row r="5" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="63"/>
-      <c r="B5" s="64"/>
+      <c r="A5" s="64"/>
+      <c r="B5" s="65"/>
       <c r="C5" s="6" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="K5" s="73"/>
-      <c r="L5" s="74"/>
+        <v>58</v>
+      </c>
+      <c r="K5" s="74"/>
+      <c r="L5" s="75"/>
     </row>
     <row r="6" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="93" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="94"/>
+      <c r="A6" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="39"/>
       <c r="C6" s="8">
         <f>SUM(C7:C71)</f>
         <v>17086</v>
@@ -1592,15 +1604,15 @@
       <c r="H6" s="35"/>
       <c r="I6" s="35"/>
       <c r="J6" s="35"/>
-      <c r="K6" s="46"/>
-      <c r="L6" s="47"/>
+      <c r="K6" s="40"/>
+      <c r="L6" s="41"/>
     </row>
     <row r="7" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="48" t="s">
-        <v>48</v>
+      <c r="A7" s="42" t="s">
+        <v>40</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C7" s="32">
         <v>10</v>
@@ -1614,13 +1626,13 @@
       <c r="H7" s="35"/>
       <c r="I7" s="35"/>
       <c r="J7" s="35"/>
-      <c r="K7" s="46"/>
-      <c r="L7" s="47"/>
+      <c r="K7" s="40"/>
+      <c r="L7" s="41"/>
     </row>
     <row r="8" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="49"/>
+      <c r="A8" s="43"/>
       <c r="B8" s="3" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="C8" s="32">
         <v>13000</v>
@@ -1634,13 +1646,13 @@
       <c r="H8" s="35"/>
       <c r="I8" s="35"/>
       <c r="J8" s="35"/>
-      <c r="K8" s="46"/>
-      <c r="L8" s="47"/>
+      <c r="K8" s="40"/>
+      <c r="L8" s="41"/>
     </row>
     <row r="9" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="55"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C9" s="9">
         <v>10</v>
@@ -1654,15 +1666,15 @@
       <c r="H9" s="35"/>
       <c r="I9" s="35"/>
       <c r="J9" s="35"/>
-      <c r="K9" s="46"/>
-      <c r="L9" s="47"/>
+      <c r="K9" s="40"/>
+      <c r="L9" s="41"/>
     </row>
     <row r="10" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="48" t="s">
-        <v>36</v>
+      <c r="A10" s="42" t="s">
+        <v>30</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C10" s="10">
         <v>64</v>
@@ -1680,9 +1692,9 @@
       <c r="L10" s="16"/>
     </row>
     <row r="11" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="49"/>
+      <c r="A11" s="43"/>
       <c r="B11" s="3" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="C11" s="10">
         <v>66</v>
@@ -1700,9 +1712,9 @@
       <c r="L11" s="16"/>
     </row>
     <row r="12" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="49"/>
+      <c r="A12" s="43"/>
       <c r="B12" s="3" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="C12" s="10">
         <v>66</v>
@@ -1720,9 +1732,9 @@
       <c r="L12" s="16"/>
     </row>
     <row r="13" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="49"/>
+      <c r="A13" s="43"/>
       <c r="B13" s="3" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C13" s="10">
         <v>31</v>
@@ -1740,9 +1752,9 @@
       <c r="L13" s="16"/>
     </row>
     <row r="14" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="49"/>
+      <c r="A14" s="43"/>
       <c r="B14" s="3" t="s">
-        <v>1</v>
+        <v>78</v>
       </c>
       <c r="C14" s="10">
         <v>66</v>
@@ -1760,9 +1772,9 @@
       <c r="L14" s="16"/>
     </row>
     <row r="15" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="49"/>
+      <c r="A15" s="43"/>
       <c r="B15" s="3" t="s">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="C15" s="10">
         <v>66</v>
@@ -1780,9 +1792,9 @@
       <c r="L15" s="16"/>
     </row>
     <row r="16" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="49"/>
+      <c r="A16" s="43"/>
       <c r="B16" s="3" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="C16" s="10">
         <v>64</v>
@@ -1798,13 +1810,13 @@
       <c r="J16" s="35"/>
       <c r="K16" s="13"/>
       <c r="L16" s="16" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="49"/>
+      <c r="A17" s="43"/>
       <c r="B17" s="3" t="s">
-        <v>19</v>
+        <v>81</v>
       </c>
       <c r="C17" s="10">
         <v>64</v>
@@ -1822,9 +1834,9 @@
       <c r="L17" s="16"/>
     </row>
     <row r="18" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="49"/>
+      <c r="A18" s="43"/>
       <c r="B18" s="3" t="s">
-        <v>47</v>
+        <v>82</v>
       </c>
       <c r="C18" s="10">
         <v>64</v>
@@ -1838,13 +1850,13 @@
       <c r="H18" s="35"/>
       <c r="I18" s="35"/>
       <c r="J18" s="35"/>
-      <c r="K18" s="50"/>
-      <c r="L18" s="47"/>
+      <c r="K18" s="80"/>
+      <c r="L18" s="41"/>
     </row>
     <row r="19" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="49"/>
+      <c r="A19" s="43"/>
       <c r="B19" s="3" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="C19" s="10">
         <v>64</v>
@@ -1862,9 +1874,9 @@
       <c r="L19" s="16"/>
     </row>
     <row r="20" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="49"/>
+      <c r="A20" s="43"/>
       <c r="B20" s="3" t="s">
-        <v>46</v>
+        <v>84</v>
       </c>
       <c r="C20" s="10">
         <v>64</v>
@@ -1882,11 +1894,11 @@
       <c r="L20" s="16"/>
     </row>
     <row r="21" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="48" t="s">
-        <v>30</v>
+      <c r="A21" s="42" t="s">
+        <v>24</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="C21" s="10">
         <v>64</v>
@@ -1900,13 +1912,13 @@
       <c r="H21" s="35"/>
       <c r="I21" s="35"/>
       <c r="J21" s="35"/>
-      <c r="K21" s="56"/>
-      <c r="L21" s="57"/>
+      <c r="K21" s="81"/>
+      <c r="L21" s="82"/>
     </row>
     <row r="22" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="49"/>
+      <c r="A22" s="43"/>
       <c r="B22" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C22" s="10">
         <v>64</v>
@@ -1920,13 +1932,13 @@
       <c r="H22" s="35"/>
       <c r="I22" s="35"/>
       <c r="J22" s="35"/>
-      <c r="K22" s="56"/>
-      <c r="L22" s="57"/>
+      <c r="K22" s="81"/>
+      <c r="L22" s="82"/>
     </row>
     <row r="23" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="49"/>
+      <c r="A23" s="43"/>
       <c r="B23" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C23" s="10">
         <v>64</v>
@@ -1940,13 +1952,13 @@
       <c r="H23" s="35"/>
       <c r="I23" s="35"/>
       <c r="J23" s="35"/>
-      <c r="K23" s="56"/>
-      <c r="L23" s="57"/>
+      <c r="K23" s="81"/>
+      <c r="L23" s="82"/>
     </row>
     <row r="24" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="49"/>
+      <c r="A24" s="43"/>
       <c r="B24" s="3" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C24" s="10">
         <v>66</v>
@@ -1960,13 +1972,13 @@
       <c r="H24" s="35"/>
       <c r="I24" s="35"/>
       <c r="J24" s="35"/>
-      <c r="K24" s="56"/>
-      <c r="L24" s="57"/>
+      <c r="K24" s="81"/>
+      <c r="L24" s="82"/>
     </row>
     <row r="25" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="49"/>
+      <c r="A25" s="43"/>
       <c r="B25" s="3" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="C25" s="10">
         <v>66</v>
@@ -1980,13 +1992,13 @@
       <c r="H25" s="35"/>
       <c r="I25" s="35"/>
       <c r="J25" s="35"/>
-      <c r="K25" s="56"/>
-      <c r="L25" s="57"/>
+      <c r="K25" s="81"/>
+      <c r="L25" s="82"/>
     </row>
     <row r="26" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="49"/>
+      <c r="A26" s="43"/>
       <c r="B26" s="3" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C26" s="10">
         <v>64</v>
@@ -2000,13 +2012,13 @@
       <c r="H26" s="35"/>
       <c r="I26" s="35"/>
       <c r="J26" s="35"/>
-      <c r="K26" s="56"/>
-      <c r="L26" s="57"/>
+      <c r="K26" s="81"/>
+      <c r="L26" s="82"/>
     </row>
     <row r="27" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="49"/>
+      <c r="A27" s="43"/>
       <c r="B27" s="3" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C27" s="10">
         <v>64</v>
@@ -2020,13 +2032,13 @@
       <c r="H27" s="35"/>
       <c r="I27" s="35"/>
       <c r="J27" s="35"/>
-      <c r="K27" s="56"/>
-      <c r="L27" s="57"/>
+      <c r="K27" s="81"/>
+      <c r="L27" s="82"/>
     </row>
     <row r="28" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="49"/>
+      <c r="A28" s="43"/>
       <c r="B28" s="3" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="C28" s="10">
         <v>64</v>
@@ -2040,13 +2052,13 @@
       <c r="H28" s="35"/>
       <c r="I28" s="35"/>
       <c r="J28" s="35"/>
-      <c r="K28" s="56"/>
-      <c r="L28" s="57"/>
+      <c r="K28" s="81"/>
+      <c r="L28" s="82"/>
     </row>
     <row r="29" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="49"/>
+      <c r="A29" s="43"/>
       <c r="B29" s="3" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C29" s="10">
         <v>33</v>
@@ -2064,9 +2076,9 @@
       <c r="L29" s="16"/>
     </row>
     <row r="30" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="49"/>
+      <c r="A30" s="43"/>
       <c r="B30" s="3" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C30" s="10">
         <v>31</v>
@@ -2084,9 +2096,9 @@
       <c r="L30" s="16"/>
     </row>
     <row r="31" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="49"/>
+      <c r="A31" s="43"/>
       <c r="B31" s="3" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C31" s="10">
         <v>33</v>
@@ -2104,9 +2116,9 @@
       <c r="L31" s="16"/>
     </row>
     <row r="32" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="49"/>
+      <c r="A32" s="43"/>
       <c r="B32" s="3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C32" s="10">
         <v>66</v>
@@ -2120,13 +2132,13 @@
       <c r="H32" s="35"/>
       <c r="I32" s="35"/>
       <c r="J32" s="35"/>
-      <c r="K32" s="50"/>
-      <c r="L32" s="47"/>
+      <c r="K32" s="80"/>
+      <c r="L32" s="41"/>
     </row>
     <row r="33" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="49"/>
+      <c r="A33" s="43"/>
       <c r="B33" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C33" s="10">
         <v>64</v>
@@ -2144,9 +2156,9 @@
       <c r="L33" s="16"/>
     </row>
     <row r="34" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="49"/>
+      <c r="A34" s="43"/>
       <c r="B34" s="3" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C34" s="10">
         <v>64</v>
@@ -2160,13 +2172,13 @@
       <c r="H34" s="35"/>
       <c r="I34" s="35"/>
       <c r="J34" s="35"/>
-      <c r="K34" s="50"/>
-      <c r="L34" s="47"/>
+      <c r="K34" s="80"/>
+      <c r="L34" s="41"/>
     </row>
     <row r="35" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="49"/>
+      <c r="A35" s="43"/>
       <c r="B35" s="3" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C35" s="10">
         <v>65</v>
@@ -2180,13 +2192,13 @@
       <c r="H35" s="35"/>
       <c r="I35" s="35"/>
       <c r="J35" s="35"/>
-      <c r="K35" s="50"/>
-      <c r="L35" s="47"/>
+      <c r="K35" s="80"/>
+      <c r="L35" s="41"/>
     </row>
     <row r="36" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="49"/>
+      <c r="A36" s="43"/>
       <c r="B36" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C36" s="10">
         <v>66</v>
@@ -2204,9 +2216,9 @@
       <c r="L36" s="16"/>
     </row>
     <row r="37" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="49"/>
+      <c r="A37" s="43"/>
       <c r="B37" s="3" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C37" s="10">
         <v>66</v>
@@ -2220,13 +2232,13 @@
       <c r="H37" s="35"/>
       <c r="I37" s="35"/>
       <c r="J37" s="35"/>
-      <c r="K37" s="50"/>
-      <c r="L37" s="47"/>
+      <c r="K37" s="80"/>
+      <c r="L37" s="41"/>
     </row>
     <row r="38" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="49"/>
+      <c r="A38" s="43"/>
       <c r="B38" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C38" s="10">
         <v>66</v>
@@ -2240,13 +2252,13 @@
       <c r="H38" s="35"/>
       <c r="I38" s="35"/>
       <c r="J38" s="35"/>
-      <c r="K38" s="50"/>
-      <c r="L38" s="47"/>
+      <c r="K38" s="80"/>
+      <c r="L38" s="41"/>
     </row>
     <row r="39" spans="1:12" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="55"/>
+      <c r="A39" s="44"/>
       <c r="B39" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C39" s="10">
         <v>33</v>
@@ -2264,67 +2276,67 @@
       <c r="L39" s="16"/>
     </row>
     <row r="40" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="83" t="s">
-        <v>57</v>
-      </c>
-      <c r="B40" s="84"/>
-      <c r="C40" s="87" t="s">
-        <v>56</v>
-      </c>
-      <c r="D40" s="88"/>
-      <c r="E40" s="89" t="s">
-        <v>64</v>
-      </c>
-      <c r="F40" s="90"/>
-      <c r="G40" s="91" t="s">
-        <v>74</v>
-      </c>
-      <c r="H40" s="92"/>
-      <c r="I40" s="91" t="s">
-        <v>72</v>
-      </c>
-      <c r="J40" s="92"/>
-      <c r="K40" s="79" t="s">
-        <v>59</v>
-      </c>
-      <c r="L40" s="80"/>
+      <c r="A40" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="B40" s="50"/>
+      <c r="C40" s="53" t="s">
+        <v>47</v>
+      </c>
+      <c r="D40" s="54"/>
+      <c r="E40" s="55" t="s">
+        <v>55</v>
+      </c>
+      <c r="F40" s="56"/>
+      <c r="G40" s="57" t="s">
+        <v>65</v>
+      </c>
+      <c r="H40" s="58"/>
+      <c r="I40" s="57" t="s">
+        <v>63</v>
+      </c>
+      <c r="J40" s="58"/>
+      <c r="K40" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="L40" s="46"/>
     </row>
     <row r="41" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="85"/>
-      <c r="B41" s="86"/>
+      <c r="A41" s="51"/>
+      <c r="B41" s="52"/>
       <c r="C41" s="19" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="D41" s="20" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="F41" s="21" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="G41" s="22" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="H41" s="22" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="I41" s="22" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="J41" s="22" t="s">
-        <v>67</v>
-      </c>
-      <c r="K41" s="81"/>
-      <c r="L41" s="82"/>
+        <v>58</v>
+      </c>
+      <c r="K41" s="47"/>
+      <c r="L41" s="48"/>
     </row>
     <row r="42" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="48" t="s">
-        <v>30</v>
+      <c r="A42" s="42" t="s">
+        <v>24</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C42" s="10">
         <v>33</v>
@@ -2342,9 +2354,9 @@
       <c r="L42" s="16"/>
     </row>
     <row r="43" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="49"/>
+      <c r="A43" s="43"/>
       <c r="B43" s="3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C43" s="10">
         <v>33</v>
@@ -2362,9 +2374,9 @@
       <c r="L43" s="16"/>
     </row>
     <row r="44" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="49"/>
+      <c r="A44" s="43"/>
       <c r="B44" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C44" s="10">
         <v>33</v>
@@ -2382,9 +2394,9 @@
       <c r="L44" s="16"/>
     </row>
     <row r="45" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="49"/>
+      <c r="A45" s="43"/>
       <c r="B45" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C45" s="10">
         <v>31</v>
@@ -2402,9 +2414,9 @@
       <c r="L45" s="16"/>
     </row>
     <row r="46" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="49"/>
+      <c r="A46" s="43"/>
       <c r="B46" s="3" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C46" s="10">
         <v>33</v>
@@ -2422,9 +2434,9 @@
       <c r="L46" s="16"/>
     </row>
     <row r="47" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="49"/>
+      <c r="A47" s="43"/>
       <c r="B47" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C47" s="10">
         <v>31</v>
@@ -2442,9 +2454,9 @@
       <c r="L47" s="16"/>
     </row>
     <row r="48" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="49"/>
+      <c r="A48" s="43"/>
       <c r="B48" s="3" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="C48" s="10">
         <v>64</v>
@@ -2458,13 +2470,13 @@
       <c r="H48" s="35"/>
       <c r="I48" s="35"/>
       <c r="J48" s="35"/>
-      <c r="K48" s="50"/>
-      <c r="L48" s="47"/>
+      <c r="K48" s="80"/>
+      <c r="L48" s="41"/>
     </row>
     <row r="49" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="49"/>
+      <c r="A49" s="43"/>
       <c r="B49" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C49" s="10">
         <v>66</v>
@@ -2478,15 +2490,15 @@
       <c r="H49" s="35"/>
       <c r="I49" s="35"/>
       <c r="J49" s="35"/>
-      <c r="K49" s="50"/>
-      <c r="L49" s="47"/>
+      <c r="K49" s="80"/>
+      <c r="L49" s="41"/>
     </row>
     <row r="50" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="48" t="s">
-        <v>33</v>
+      <c r="A50" s="42" t="s">
+        <v>27</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C50" s="10">
         <v>2</v>
@@ -2494,7 +2506,7 @@
       <c r="D50" s="28">
         <v>2400</v>
       </c>
-      <c r="E50" s="35"/>
+      <c r="E50" s="95"/>
       <c r="F50" s="35"/>
       <c r="G50" s="35"/>
       <c r="H50" s="35"/>
@@ -2504,9 +2516,9 @@
       <c r="L50" s="16"/>
     </row>
     <row r="51" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="49"/>
+      <c r="A51" s="43"/>
       <c r="B51" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C51" s="10">
         <v>1</v>
@@ -2524,9 +2536,9 @@
       <c r="L51" s="16"/>
     </row>
     <row r="52" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="49"/>
+      <c r="A52" s="43"/>
       <c r="B52" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C52" s="10">
         <v>1</v>
@@ -2544,9 +2556,9 @@
       <c r="L52" s="16"/>
     </row>
     <row r="53" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="49"/>
+      <c r="A53" s="43"/>
       <c r="B53" s="14" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C53" s="12">
         <v>137</v>
@@ -2560,13 +2572,13 @@
       <c r="H53" s="35"/>
       <c r="I53" s="35"/>
       <c r="J53" s="35"/>
-      <c r="K53" s="51"/>
-      <c r="L53" s="52"/>
+      <c r="K53" s="83"/>
+      <c r="L53" s="84"/>
     </row>
     <row r="54" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="49"/>
+      <c r="A54" s="43"/>
       <c r="B54" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C54" s="12">
         <v>1</v>
@@ -2580,15 +2592,15 @@
       <c r="H54" s="35"/>
       <c r="I54" s="35"/>
       <c r="J54" s="35"/>
-      <c r="K54" s="46" t="s">
-        <v>65</v>
-      </c>
-      <c r="L54" s="47"/>
+      <c r="K54" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="L54" s="41"/>
     </row>
     <row r="55" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="49"/>
+      <c r="A55" s="43"/>
       <c r="B55" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C55" s="12">
         <v>10</v>
@@ -2602,13 +2614,13 @@
       <c r="H55" s="35"/>
       <c r="I55" s="35"/>
       <c r="J55" s="35"/>
-      <c r="K55" s="46"/>
-      <c r="L55" s="47"/>
+      <c r="K55" s="40"/>
+      <c r="L55" s="41"/>
     </row>
     <row r="56" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="49"/>
+      <c r="A56" s="43"/>
       <c r="B56" s="15" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C56" s="23">
         <v>1</v>
@@ -2622,15 +2634,15 @@
       <c r="H56" s="37"/>
       <c r="I56" s="35"/>
       <c r="J56" s="35"/>
-      <c r="K56" s="53"/>
-      <c r="L56" s="54"/>
+      <c r="K56" s="85"/>
+      <c r="L56" s="86"/>
     </row>
     <row r="57" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="48" t="s">
-        <v>37</v>
+      <c r="A57" s="42" t="s">
+        <v>31</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C57" s="24">
         <v>300</v>
@@ -2648,9 +2660,9 @@
       <c r="L57" s="16"/>
     </row>
     <row r="58" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="49"/>
+      <c r="A58" s="43"/>
       <c r="B58" s="3" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="C58" s="24">
         <v>250</v>
@@ -2668,9 +2680,9 @@
       <c r="L58" s="16"/>
     </row>
     <row r="59" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="49"/>
+      <c r="A59" s="43"/>
       <c r="B59" s="25" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="C59" s="24">
         <v>300</v>
@@ -2684,13 +2696,13 @@
       <c r="H59" s="35"/>
       <c r="I59" s="35"/>
       <c r="J59" s="35"/>
-      <c r="K59" s="46"/>
-      <c r="L59" s="47"/>
+      <c r="K59" s="40"/>
+      <c r="L59" s="41"/>
     </row>
     <row r="60" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="49"/>
+      <c r="A60" s="43"/>
       <c r="B60" s="25" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="C60" s="24">
         <v>250</v>
@@ -2708,9 +2720,9 @@
       <c r="L60" s="16"/>
     </row>
     <row r="61" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="49"/>
+      <c r="A61" s="43"/>
       <c r="B61" s="25" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" s="24">
         <v>300</v>
@@ -2724,13 +2736,13 @@
       <c r="H61" s="35"/>
       <c r="I61" s="35"/>
       <c r="J61" s="35"/>
-      <c r="K61" s="46"/>
-      <c r="L61" s="47"/>
+      <c r="K61" s="40"/>
+      <c r="L61" s="41"/>
     </row>
     <row r="62" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="55"/>
+      <c r="A62" s="44"/>
       <c r="B62" s="25" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="C62" s="24">
         <v>300</v>
@@ -2744,15 +2756,15 @@
       <c r="H62" s="35"/>
       <c r="I62" s="35"/>
       <c r="J62" s="35"/>
-      <c r="K62" s="46"/>
-      <c r="L62" s="47"/>
+      <c r="K62" s="40"/>
+      <c r="L62" s="41"/>
     </row>
     <row r="63" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C63" s="9">
         <v>4</v>
@@ -2770,11 +2782,11 @@
       <c r="L63" s="16"/>
     </row>
     <row r="64" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="48" t="s">
-        <v>20</v>
+      <c r="A64" s="42" t="s">
+        <v>16</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C64" s="9">
         <v>100</v>
@@ -2788,13 +2800,13 @@
       <c r="H64" s="35"/>
       <c r="I64" s="35"/>
       <c r="J64" s="35"/>
-      <c r="K64" s="50"/>
-      <c r="L64" s="47"/>
+      <c r="K64" s="80"/>
+      <c r="L64" s="41"/>
     </row>
     <row r="65" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="49"/>
+      <c r="A65" s="43"/>
       <c r="B65" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C65" s="9">
         <v>1</v>
@@ -2808,13 +2820,13 @@
       <c r="H65" s="35"/>
       <c r="I65" s="35"/>
       <c r="J65" s="35"/>
-      <c r="K65" s="46"/>
-      <c r="L65" s="47"/>
+      <c r="K65" s="40"/>
+      <c r="L65" s="41"/>
     </row>
     <row r="66" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="49"/>
+      <c r="A66" s="43"/>
       <c r="B66" s="3" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C66" s="9">
         <v>1</v>
@@ -2832,9 +2844,9 @@
       <c r="L66" s="16"/>
     </row>
     <row r="67" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="55"/>
+      <c r="A67" s="44"/>
       <c r="B67" s="36" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C67" s="9">
         <v>1</v>
@@ -2852,195 +2864,174 @@
       <c r="L67" s="16"/>
     </row>
     <row r="68" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="B68" s="38"/>
-      <c r="C68" s="39"/>
-      <c r="D68" s="39"/>
-      <c r="E68" s="39"/>
-      <c r="F68" s="39"/>
-      <c r="G68" s="39"/>
-      <c r="H68" s="39"/>
-      <c r="I68" s="39"/>
-      <c r="J68" s="39"/>
-      <c r="K68" s="39"/>
-      <c r="L68" s="39"/>
+      <c r="A68" s="87" t="s">
+        <v>22</v>
+      </c>
+      <c r="B68" s="87"/>
+      <c r="C68" s="88"/>
+      <c r="D68" s="88"/>
+      <c r="E68" s="88"/>
+      <c r="F68" s="88"/>
+      <c r="G68" s="88"/>
+      <c r="H68" s="88"/>
+      <c r="I68" s="88"/>
+      <c r="J68" s="88"/>
+      <c r="K68" s="88"/>
+      <c r="L68" s="88"/>
     </row>
     <row r="69" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="38"/>
-      <c r="B69" s="38"/>
-      <c r="C69" s="39"/>
-      <c r="D69" s="39"/>
-      <c r="E69" s="39"/>
-      <c r="F69" s="39"/>
-      <c r="G69" s="39"/>
-      <c r="H69" s="39"/>
-      <c r="I69" s="39"/>
-      <c r="J69" s="39"/>
-      <c r="K69" s="39"/>
-      <c r="L69" s="39"/>
+      <c r="A69" s="87"/>
+      <c r="B69" s="87"/>
+      <c r="C69" s="88"/>
+      <c r="D69" s="88"/>
+      <c r="E69" s="88"/>
+      <c r="F69" s="88"/>
+      <c r="G69" s="88"/>
+      <c r="H69" s="88"/>
+      <c r="I69" s="88"/>
+      <c r="J69" s="88"/>
+      <c r="K69" s="88"/>
+      <c r="L69" s="88"/>
     </row>
     <row r="70" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="38"/>
-      <c r="B70" s="38"/>
-      <c r="C70" s="39"/>
-      <c r="D70" s="39"/>
-      <c r="E70" s="39"/>
-      <c r="F70" s="39"/>
-      <c r="G70" s="39"/>
-      <c r="H70" s="39"/>
-      <c r="I70" s="39"/>
-      <c r="J70" s="39"/>
-      <c r="K70" s="39"/>
-      <c r="L70" s="39"/>
+      <c r="A70" s="87"/>
+      <c r="B70" s="87"/>
+      <c r="C70" s="88"/>
+      <c r="D70" s="88"/>
+      <c r="E70" s="88"/>
+      <c r="F70" s="88"/>
+      <c r="G70" s="88"/>
+      <c r="H70" s="88"/>
+      <c r="I70" s="88"/>
+      <c r="J70" s="88"/>
+      <c r="K70" s="88"/>
+      <c r="L70" s="88"/>
     </row>
     <row r="71" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="38"/>
-      <c r="B71" s="38"/>
-      <c r="C71" s="39"/>
-      <c r="D71" s="39"/>
-      <c r="E71" s="39"/>
-      <c r="F71" s="39"/>
-      <c r="G71" s="39"/>
-      <c r="H71" s="39"/>
-      <c r="I71" s="39"/>
-      <c r="J71" s="39"/>
-      <c r="K71" s="39"/>
-      <c r="L71" s="39"/>
+      <c r="A71" s="87"/>
+      <c r="B71" s="87"/>
+      <c r="C71" s="88"/>
+      <c r="D71" s="88"/>
+      <c r="E71" s="88"/>
+      <c r="F71" s="88"/>
+      <c r="G71" s="88"/>
+      <c r="H71" s="88"/>
+      <c r="I71" s="88"/>
+      <c r="J71" s="88"/>
+      <c r="K71" s="88"/>
+      <c r="L71" s="88"/>
     </row>
     <row r="72" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="38"/>
-      <c r="B72" s="38"/>
-      <c r="C72" s="39"/>
-      <c r="D72" s="39"/>
-      <c r="E72" s="39"/>
-      <c r="F72" s="39"/>
-      <c r="G72" s="39"/>
-      <c r="H72" s="39"/>
-      <c r="I72" s="39"/>
-      <c r="J72" s="39"/>
-      <c r="K72" s="39"/>
-      <c r="L72" s="39"/>
+      <c r="A72" s="87"/>
+      <c r="B72" s="87"/>
+      <c r="C72" s="88"/>
+      <c r="D72" s="88"/>
+      <c r="E72" s="88"/>
+      <c r="F72" s="88"/>
+      <c r="G72" s="88"/>
+      <c r="H72" s="88"/>
+      <c r="I72" s="88"/>
+      <c r="J72" s="88"/>
+      <c r="K72" s="88"/>
+      <c r="L72" s="88"/>
     </row>
     <row r="73" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="38"/>
-      <c r="B73" s="38"/>
-      <c r="C73" s="39"/>
-      <c r="D73" s="39"/>
-      <c r="E73" s="39"/>
-      <c r="F73" s="39"/>
-      <c r="G73" s="39"/>
-      <c r="H73" s="39"/>
-      <c r="I73" s="39"/>
-      <c r="J73" s="39"/>
-      <c r="K73" s="39"/>
-      <c r="L73" s="39"/>
+      <c r="A73" s="87"/>
+      <c r="B73" s="87"/>
+      <c r="C73" s="88"/>
+      <c r="D73" s="88"/>
+      <c r="E73" s="88"/>
+      <c r="F73" s="88"/>
+      <c r="G73" s="88"/>
+      <c r="H73" s="88"/>
+      <c r="I73" s="88"/>
+      <c r="J73" s="88"/>
+      <c r="K73" s="88"/>
+      <c r="L73" s="88"/>
     </row>
     <row r="74" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="38"/>
-      <c r="B74" s="38"/>
-      <c r="C74" s="39"/>
-      <c r="D74" s="39"/>
-      <c r="E74" s="39"/>
-      <c r="F74" s="39"/>
-      <c r="G74" s="39"/>
-      <c r="H74" s="39"/>
-      <c r="I74" s="39"/>
-      <c r="J74" s="39"/>
-      <c r="K74" s="39"/>
-      <c r="L74" s="39"/>
+      <c r="A74" s="87"/>
+      <c r="B74" s="87"/>
+      <c r="C74" s="88"/>
+      <c r="D74" s="88"/>
+      <c r="E74" s="88"/>
+      <c r="F74" s="88"/>
+      <c r="G74" s="88"/>
+      <c r="H74" s="88"/>
+      <c r="I74" s="88"/>
+      <c r="J74" s="88"/>
+      <c r="K74" s="88"/>
+      <c r="L74" s="88"/>
     </row>
     <row r="75" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="38"/>
-      <c r="B75" s="38"/>
-      <c r="C75" s="39"/>
-      <c r="D75" s="39"/>
-      <c r="E75" s="39"/>
-      <c r="F75" s="39"/>
-      <c r="G75" s="39"/>
-      <c r="H75" s="39"/>
-      <c r="I75" s="39"/>
-      <c r="J75" s="39"/>
-      <c r="K75" s="39"/>
-      <c r="L75" s="39"/>
+      <c r="A75" s="87"/>
+      <c r="B75" s="87"/>
+      <c r="C75" s="88"/>
+      <c r="D75" s="88"/>
+      <c r="E75" s="88"/>
+      <c r="F75" s="88"/>
+      <c r="G75" s="88"/>
+      <c r="H75" s="88"/>
+      <c r="I75" s="88"/>
+      <c r="J75" s="88"/>
+      <c r="K75" s="88"/>
+      <c r="L75" s="88"/>
     </row>
     <row r="76" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="38"/>
-      <c r="B76" s="38"/>
-      <c r="C76" s="39"/>
-      <c r="D76" s="39"/>
-      <c r="E76" s="39"/>
-      <c r="F76" s="39"/>
-      <c r="G76" s="39"/>
-      <c r="H76" s="39"/>
-      <c r="I76" s="39"/>
-      <c r="J76" s="39"/>
-      <c r="K76" s="39"/>
-      <c r="L76" s="39"/>
+      <c r="A76" s="87"/>
+      <c r="B76" s="87"/>
+      <c r="C76" s="88"/>
+      <c r="D76" s="88"/>
+      <c r="E76" s="88"/>
+      <c r="F76" s="88"/>
+      <c r="G76" s="88"/>
+      <c r="H76" s="88"/>
+      <c r="I76" s="88"/>
+      <c r="J76" s="88"/>
+      <c r="K76" s="88"/>
+      <c r="L76" s="88"/>
     </row>
     <row r="77" spans="1:12" s="34" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="B77" s="38"/>
-      <c r="C77" s="40"/>
-      <c r="D77" s="41"/>
-      <c r="E77" s="41"/>
-      <c r="F77" s="41"/>
-      <c r="G77" s="41"/>
-      <c r="H77" s="41"/>
-      <c r="I77" s="41"/>
-      <c r="J77" s="41"/>
-      <c r="K77" s="41"/>
-      <c r="L77" s="42"/>
+      <c r="A77" s="87" t="s">
+        <v>50</v>
+      </c>
+      <c r="B77" s="87"/>
+      <c r="C77" s="89"/>
+      <c r="D77" s="90"/>
+      <c r="E77" s="90"/>
+      <c r="F77" s="90"/>
+      <c r="G77" s="90"/>
+      <c r="H77" s="90"/>
+      <c r="I77" s="90"/>
+      <c r="J77" s="90"/>
+      <c r="K77" s="90"/>
+      <c r="L77" s="91"/>
     </row>
     <row r="78" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="38"/>
-      <c r="B78" s="38"/>
-      <c r="C78" s="43"/>
-      <c r="D78" s="44"/>
-      <c r="E78" s="44"/>
-      <c r="F78" s="44"/>
-      <c r="G78" s="44"/>
-      <c r="H78" s="44"/>
-      <c r="I78" s="44"/>
-      <c r="J78" s="44"/>
-      <c r="K78" s="44"/>
-      <c r="L78" s="45"/>
+      <c r="A78" s="87"/>
+      <c r="B78" s="87"/>
+      <c r="C78" s="92"/>
+      <c r="D78" s="93"/>
+      <c r="E78" s="93"/>
+      <c r="F78" s="93"/>
+      <c r="G78" s="93"/>
+      <c r="H78" s="93"/>
+      <c r="I78" s="93"/>
+      <c r="J78" s="93"/>
+      <c r="K78" s="93"/>
+      <c r="L78" s="94"/>
     </row>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="K40:L41"/>
-    <mergeCell ref="A57:A62"/>
-    <mergeCell ref="K59:L59"/>
-    <mergeCell ref="K61:L61"/>
-    <mergeCell ref="K62:L62"/>
-    <mergeCell ref="A40:B41"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L5"/>
-    <mergeCell ref="A1:F2"/>
-    <mergeCell ref="G1:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="K55:L55"/>
+    <mergeCell ref="K56:L56"/>
+    <mergeCell ref="A68:B76"/>
+    <mergeCell ref="C68:L76"/>
+    <mergeCell ref="A77:B78"/>
+    <mergeCell ref="C77:L78"/>
+    <mergeCell ref="K65:L65"/>
+    <mergeCell ref="A64:A67"/>
+    <mergeCell ref="K64:L64"/>
     <mergeCell ref="A10:A20"/>
     <mergeCell ref="K18:L18"/>
     <mergeCell ref="A21:A39"/>
@@ -3057,21 +3048,42 @@
     <mergeCell ref="K35:L35"/>
     <mergeCell ref="K37:L37"/>
     <mergeCell ref="K38:L38"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L5"/>
+    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="G1:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="K40:L41"/>
+    <mergeCell ref="A57:A62"/>
+    <mergeCell ref="K59:L59"/>
+    <mergeCell ref="K61:L61"/>
+    <mergeCell ref="K62:L62"/>
+    <mergeCell ref="A40:B41"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="I40:J40"/>
     <mergeCell ref="A42:A49"/>
     <mergeCell ref="K48:L48"/>
     <mergeCell ref="K49:L49"/>
     <mergeCell ref="A50:A56"/>
     <mergeCell ref="K53:L53"/>
     <mergeCell ref="K54:L54"/>
-    <mergeCell ref="K55:L55"/>
-    <mergeCell ref="K56:L56"/>
-    <mergeCell ref="A68:B76"/>
-    <mergeCell ref="C68:L76"/>
-    <mergeCell ref="A77:B78"/>
-    <mergeCell ref="C77:L78"/>
-    <mergeCell ref="K65:L65"/>
-    <mergeCell ref="A64:A67"/>
-    <mergeCell ref="K64:L64"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="K9:L9"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>